<commit_message>
convert to english button
</commit_message>
<xml_diff>
--- a/data/results/ivr_responses.xlsx
+++ b/data/results/ivr_responses.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,65 +464,10 @@
           <t>q6</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>q7</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>q8</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>q9</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>q10</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>q11</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>q12</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>q13</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>q14</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>q15</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>q16</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>q17</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>111</v>
+        <v>3</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -551,116 +496,49 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Wote wawili</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Marafiki</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+          <t>Mke pekee</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>111</t>
-        </is>
+      <c r="A3" t="n">
+        <v>5</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kuhamia sehemu nyingine</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Mume na mama mkwe</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Kuzungumza kuhusu afya na kupanga watoto</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Uvimbe kwenye kizazi (fibroidi)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Njia zote ni za kudumu</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Mume pekee</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
+          <t>Kufungua mkahawa</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kufungua mkahawa</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>Marafiki</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Mungu ndiye anaamua jinsia ya mtoto</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Anamuunga mkono</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Kuonyesha umuhimu wa maamuzi ya mwanamke</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Aliondoka ndoani</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Wanasema watoto wa kike hawawezi kusaidia</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Akae nyumbani</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Familia na elimu vinaweza kwenda pamoja</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Mwanamke anaweza kupanga maisha yake akipata msaada</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Nyingine</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Nyingine</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mado ni mjamzito</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
english translation and exxport button for both things are added
</commit_message>
<xml_diff>
--- a/data/results/ivr_responses.xlsx
+++ b/data/results/ivr_responses.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,10 +464,20 @@
           <t>q6</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>q7</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>q8</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -496,24 +506,60 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Mke pekee</t>
+          <t>Wote wawili</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Marafiki</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Mungu ndiye anaamua jinsia ya mtoto</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kufungua mkahawa</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+          <t>Kumaliza masomo ya unesi</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Marafiki</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mado ni mjamzito</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Uvimbe kwenye kizazi (fibroidi)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Njia zote ni za kudumu</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Wote wawili</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Mitandao ya kijamii (Kwa mfano Facebook, Instagram, X)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -528,17 +574,39 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Mume na mama mkwe</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Kuchagua jinsia ya mtoto</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Presha ya damu</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Njia nyingi unaweza kuachwa baadaye</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Mume pekee</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>Marafiki</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Mado ni mjamzito</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Mungu ndiye anaamua jinsia ya mtoto</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>